<commit_message>
second stable pypf package commit
</commit_message>
<xml_diff>
--- a/data/psy.prx.xlsx
+++ b/data/psy.prx.xlsx
@@ -1,27 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schva\Prog\mypy\nets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schva\Prog\py_proj\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E1C723-7C2C-4B96-A7C3-C9FA3182B5DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5856A160-2155-4298-BD36-E90AE71C04A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9495" yWindow="0" windowWidth="9810" windowHeight="7425" xr2:uid="{7F0295F9-5E1B-42CA-8214-BAD83C5FD4BA}"/>
+    <workbookView xWindow="-21375" yWindow="885" windowWidth="19410" windowHeight="14370" xr2:uid="{7F0295F9-5E1B-42CA-8214-BAD83C5FD4BA}"/>
   </bookViews>
   <sheets>
     <sheet name="colterms" sheetId="1" r:id="rId1"/>
-    <sheet name="nocolterms" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="25">
   <si>
     <t>living thing</t>
   </si>
@@ -958,6 +957,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8236EA58-9DD5-425F-A41E-2090E861D3F2}">
   <dimension ref="A1:Z26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="5.85546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="3.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="B1" t="s">
@@ -3033,2020 +3059,6 @@
         <v>32</v>
       </c>
       <c r="Z26">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80E7C07A-DEC4-48A0-9E30-DFD73955F729}">
-  <dimension ref="A1:Z25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="26" width="3" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1">
-        <v>0</v>
-      </c>
-      <c r="C1">
-        <v>13</v>
-      </c>
-      <c r="D1">
-        <v>29</v>
-      </c>
-      <c r="E1">
-        <v>18</v>
-      </c>
-      <c r="F1">
-        <v>51</v>
-      </c>
-      <c r="G1">
-        <v>23</v>
-      </c>
-      <c r="H1">
-        <v>17</v>
-      </c>
-      <c r="I1">
-        <v>18</v>
-      </c>
-      <c r="J1">
-        <v>45</v>
-      </c>
-      <c r="K1">
-        <v>15</v>
-      </c>
-      <c r="L1">
-        <v>15</v>
-      </c>
-      <c r="M1">
-        <v>22</v>
-      </c>
-      <c r="N1">
-        <v>41</v>
-      </c>
-      <c r="O1">
-        <v>48</v>
-      </c>
-      <c r="P1">
-        <v>23</v>
-      </c>
-      <c r="Q1">
-        <v>20</v>
-      </c>
-      <c r="R1">
-        <v>33</v>
-      </c>
-      <c r="S1">
-        <v>18</v>
-      </c>
-      <c r="T1">
-        <v>28</v>
-      </c>
-      <c r="U1">
-        <v>22</v>
-      </c>
-      <c r="V1">
-        <v>30</v>
-      </c>
-      <c r="W1">
-        <v>31</v>
-      </c>
-      <c r="X1">
-        <v>45</v>
-      </c>
-      <c r="Y1">
-        <v>35</v>
-      </c>
-      <c r="Z1">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>13</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>26</v>
-      </c>
-      <c r="E2">
-        <v>25</v>
-      </c>
-      <c r="F2">
-        <v>44</v>
-      </c>
-      <c r="G2">
-        <v>34</v>
-      </c>
-      <c r="H2">
-        <v>23</v>
-      </c>
-      <c r="I2">
-        <v>15</v>
-      </c>
-      <c r="J2">
-        <v>33</v>
-      </c>
-      <c r="K2">
-        <v>13</v>
-      </c>
-      <c r="L2">
-        <v>11</v>
-      </c>
-      <c r="M2">
-        <v>28</v>
-      </c>
-      <c r="N2">
-        <v>31</v>
-      </c>
-      <c r="O2">
-        <v>35</v>
-      </c>
-      <c r="P2">
-        <v>28</v>
-      </c>
-      <c r="Q2">
-        <v>47</v>
-      </c>
-      <c r="R2">
-        <v>65</v>
-      </c>
-      <c r="S2">
-        <v>49</v>
-      </c>
-      <c r="T2">
-        <v>58</v>
-      </c>
-      <c r="U2">
-        <v>49</v>
-      </c>
-      <c r="V2">
-        <v>64</v>
-      </c>
-      <c r="W2">
-        <v>55</v>
-      </c>
-      <c r="X2">
-        <v>53</v>
-      </c>
-      <c r="Y2">
-        <v>69</v>
-      </c>
-      <c r="Z2">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>29</v>
-      </c>
-      <c r="C3">
-        <v>26</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>47</v>
-      </c>
-      <c r="F3">
-        <v>54</v>
-      </c>
-      <c r="G3">
-        <v>43</v>
-      </c>
-      <c r="H3">
-        <v>43</v>
-      </c>
-      <c r="I3">
-        <v>27</v>
-      </c>
-      <c r="J3">
-        <v>55</v>
-      </c>
-      <c r="K3">
-        <v>39</v>
-      </c>
-      <c r="L3">
-        <v>37</v>
-      </c>
-      <c r="M3">
-        <v>35</v>
-      </c>
-      <c r="N3">
-        <v>48</v>
-      </c>
-      <c r="O3">
-        <v>54</v>
-      </c>
-      <c r="P3">
-        <v>51</v>
-      </c>
-      <c r="Q3">
-        <v>73</v>
-      </c>
-      <c r="R3">
-        <v>64</v>
-      </c>
-      <c r="S3">
-        <v>74</v>
-      </c>
-      <c r="T3">
-        <v>76</v>
-      </c>
-      <c r="U3">
-        <v>70</v>
-      </c>
-      <c r="V3">
-        <v>47</v>
-      </c>
-      <c r="W3">
-        <v>78</v>
-      </c>
-      <c r="X3">
-        <v>35</v>
-      </c>
-      <c r="Y3">
-        <v>76</v>
-      </c>
-      <c r="Z3">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>18</v>
-      </c>
-      <c r="C4">
-        <v>25</v>
-      </c>
-      <c r="D4">
-        <v>47</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>8</v>
-      </c>
-      <c r="G4">
-        <v>12</v>
-      </c>
-      <c r="H4">
-        <v>18</v>
-      </c>
-      <c r="I4">
-        <v>36</v>
-      </c>
-      <c r="J4">
-        <v>65</v>
-      </c>
-      <c r="K4">
-        <v>35</v>
-      </c>
-      <c r="L4">
-        <v>41</v>
-      </c>
-      <c r="M4">
-        <v>22</v>
-      </c>
-      <c r="N4">
-        <v>73</v>
-      </c>
-      <c r="O4">
-        <v>72</v>
-      </c>
-      <c r="P4">
-        <v>48</v>
-      </c>
-      <c r="Q4">
-        <v>48</v>
-      </c>
-      <c r="R4">
-        <v>53</v>
-      </c>
-      <c r="S4">
-        <v>26</v>
-      </c>
-      <c r="T4">
-        <v>46</v>
-      </c>
-      <c r="U4">
-        <v>50</v>
-      </c>
-      <c r="V4">
-        <v>48</v>
-      </c>
-      <c r="W4">
-        <v>54</v>
-      </c>
-      <c r="X4">
-        <v>45</v>
-      </c>
-      <c r="Y4">
-        <v>65</v>
-      </c>
-      <c r="Z4">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>51</v>
-      </c>
-      <c r="C5">
-        <v>44</v>
-      </c>
-      <c r="D5">
-        <v>54</v>
-      </c>
-      <c r="E5">
-        <v>8</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>17</v>
-      </c>
-      <c r="H5">
-        <v>15</v>
-      </c>
-      <c r="I5">
-        <v>62</v>
-      </c>
-      <c r="J5">
-        <v>36</v>
-      </c>
-      <c r="K5">
-        <v>73</v>
-      </c>
-      <c r="L5">
-        <v>73</v>
-      </c>
-      <c r="M5">
-        <v>70</v>
-      </c>
-      <c r="N5">
-        <v>56</v>
-      </c>
-      <c r="O5">
-        <v>56</v>
-      </c>
-      <c r="P5">
-        <v>72</v>
-      </c>
-      <c r="Q5">
-        <v>73</v>
-      </c>
-      <c r="R5">
-        <v>53</v>
-      </c>
-      <c r="S5">
-        <v>67</v>
-      </c>
-      <c r="T5">
-        <v>62</v>
-      </c>
-      <c r="U5">
-        <v>62</v>
-      </c>
-      <c r="V5">
-        <v>73</v>
-      </c>
-      <c r="W5">
-        <v>68</v>
-      </c>
-      <c r="X5">
-        <v>45</v>
-      </c>
-      <c r="Y5">
-        <v>59</v>
-      </c>
-      <c r="Z5">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6">
-        <v>23</v>
-      </c>
-      <c r="C6">
-        <v>34</v>
-      </c>
-      <c r="D6">
-        <v>43</v>
-      </c>
-      <c r="E6">
-        <v>12</v>
-      </c>
-      <c r="F6">
-        <v>17</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>27</v>
-      </c>
-      <c r="I6">
-        <v>47</v>
-      </c>
-      <c r="J6">
-        <v>67</v>
-      </c>
-      <c r="K6">
-        <v>44</v>
-      </c>
-      <c r="L6">
-        <v>42</v>
-      </c>
-      <c r="M6">
-        <v>32</v>
-      </c>
-      <c r="N6">
-        <v>65</v>
-      </c>
-      <c r="O6">
-        <v>74</v>
-      </c>
-      <c r="P6">
-        <v>48</v>
-      </c>
-      <c r="Q6">
-        <v>55</v>
-      </c>
-      <c r="R6">
-        <v>55</v>
-      </c>
-      <c r="S6">
-        <v>26</v>
-      </c>
-      <c r="T6">
-        <v>37</v>
-      </c>
-      <c r="U6">
-        <v>47</v>
-      </c>
-      <c r="V6">
-        <v>49</v>
-      </c>
-      <c r="W6">
-        <v>53</v>
-      </c>
-      <c r="X6">
-        <v>39</v>
-      </c>
-      <c r="Y6">
-        <v>74</v>
-      </c>
-      <c r="Z6">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>17</v>
-      </c>
-      <c r="C7">
-        <v>23</v>
-      </c>
-      <c r="D7">
-        <v>43</v>
-      </c>
-      <c r="E7">
-        <v>18</v>
-      </c>
-      <c r="F7">
-        <v>15</v>
-      </c>
-      <c r="G7">
-        <v>27</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>47</v>
-      </c>
-      <c r="J7">
-        <v>67</v>
-      </c>
-      <c r="K7">
-        <v>41</v>
-      </c>
-      <c r="L7">
-        <v>41</v>
-      </c>
-      <c r="M7">
-        <v>45</v>
-      </c>
-      <c r="N7">
-        <v>68</v>
-      </c>
-      <c r="O7">
-        <v>76</v>
-      </c>
-      <c r="P7">
-        <v>47</v>
-      </c>
-      <c r="Q7">
-        <v>63</v>
-      </c>
-      <c r="R7">
-        <v>72</v>
-      </c>
-      <c r="S7">
-        <v>58</v>
-      </c>
-      <c r="T7">
-        <v>57</v>
-      </c>
-      <c r="U7">
-        <v>60</v>
-      </c>
-      <c r="V7">
-        <v>63</v>
-      </c>
-      <c r="W7">
-        <v>67</v>
-      </c>
-      <c r="X7">
-        <v>55</v>
-      </c>
-      <c r="Y7">
-        <v>78</v>
-      </c>
-      <c r="Z7">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8">
-        <v>18</v>
-      </c>
-      <c r="C8">
-        <v>15</v>
-      </c>
-      <c r="D8">
-        <v>27</v>
-      </c>
-      <c r="E8">
-        <v>36</v>
-      </c>
-      <c r="F8">
-        <v>62</v>
-      </c>
-      <c r="G8">
-        <v>47</v>
-      </c>
-      <c r="H8">
-        <v>47</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8">
-        <v>33</v>
-      </c>
-      <c r="K8">
-        <v>20</v>
-      </c>
-      <c r="L8">
-        <v>24</v>
-      </c>
-      <c r="M8">
-        <v>24</v>
-      </c>
-      <c r="N8">
-        <v>35</v>
-      </c>
-      <c r="O8">
-        <v>35</v>
-      </c>
-      <c r="P8">
-        <v>49</v>
-      </c>
-      <c r="Q8">
-        <v>54</v>
-      </c>
-      <c r="R8">
-        <v>59</v>
-      </c>
-      <c r="S8">
-        <v>54</v>
-      </c>
-      <c r="T8">
-        <v>60</v>
-      </c>
-      <c r="U8">
-        <v>60</v>
-      </c>
-      <c r="V8">
-        <v>63</v>
-      </c>
-      <c r="W8">
-        <v>63</v>
-      </c>
-      <c r="X8">
-        <v>56</v>
-      </c>
-      <c r="Y8">
-        <v>72</v>
-      </c>
-      <c r="Z8">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>45</v>
-      </c>
-      <c r="C9">
-        <v>33</v>
-      </c>
-      <c r="D9">
-        <v>55</v>
-      </c>
-      <c r="E9">
-        <v>65</v>
-      </c>
-      <c r="F9">
-        <v>36</v>
-      </c>
-      <c r="G9">
-        <v>67</v>
-      </c>
-      <c r="H9">
-        <v>67</v>
-      </c>
-      <c r="I9">
-        <v>33</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>20</v>
-      </c>
-      <c r="L9">
-        <v>44</v>
-      </c>
-      <c r="M9">
-        <v>47</v>
-      </c>
-      <c r="N9">
-        <v>49</v>
-      </c>
-      <c r="O9">
-        <v>53</v>
-      </c>
-      <c r="P9">
-        <v>80</v>
-      </c>
-      <c r="Q9">
-        <v>64</v>
-      </c>
-      <c r="R9">
-        <v>55</v>
-      </c>
-      <c r="S9">
-        <v>71</v>
-      </c>
-      <c r="T9">
-        <v>69</v>
-      </c>
-      <c r="U9">
-        <v>73</v>
-      </c>
-      <c r="V9">
-        <v>75</v>
-      </c>
-      <c r="W9">
-        <v>72</v>
-      </c>
-      <c r="X9">
-        <v>49</v>
-      </c>
-      <c r="Y9">
-        <v>75</v>
-      </c>
-      <c r="Z9">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>15</v>
-      </c>
-      <c r="C10">
-        <v>13</v>
-      </c>
-      <c r="D10">
-        <v>39</v>
-      </c>
-      <c r="E10">
-        <v>35</v>
-      </c>
-      <c r="F10">
-        <v>73</v>
-      </c>
-      <c r="G10">
-        <v>44</v>
-      </c>
-      <c r="H10">
-        <v>41</v>
-      </c>
-      <c r="I10">
-        <v>20</v>
-      </c>
-      <c r="J10">
-        <v>20</v>
-      </c>
-      <c r="K10">
-        <v>0</v>
-      </c>
-      <c r="L10">
-        <v>35</v>
-      </c>
-      <c r="M10">
-        <v>43</v>
-      </c>
-      <c r="N10">
-        <v>66</v>
-      </c>
-      <c r="O10">
-        <v>61</v>
-      </c>
-      <c r="P10">
-        <v>42</v>
-      </c>
-      <c r="Q10">
-        <v>57</v>
-      </c>
-      <c r="R10">
-        <v>68</v>
-      </c>
-      <c r="S10">
-        <v>46</v>
-      </c>
-      <c r="T10">
-        <v>57</v>
-      </c>
-      <c r="U10">
-        <v>63</v>
-      </c>
-      <c r="V10">
-        <v>64</v>
-      </c>
-      <c r="W10">
-        <v>57</v>
-      </c>
-      <c r="X10">
-        <v>51</v>
-      </c>
-      <c r="Y10">
-        <v>77</v>
-      </c>
-      <c r="Z10">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11">
-        <v>15</v>
-      </c>
-      <c r="C11">
-        <v>11</v>
-      </c>
-      <c r="D11">
-        <v>37</v>
-      </c>
-      <c r="E11">
-        <v>41</v>
-      </c>
-      <c r="F11">
-        <v>73</v>
-      </c>
-      <c r="G11">
-        <v>42</v>
-      </c>
-      <c r="H11">
-        <v>41</v>
-      </c>
-      <c r="I11">
-        <v>24</v>
-      </c>
-      <c r="J11">
-        <v>44</v>
-      </c>
-      <c r="K11">
-        <v>35</v>
-      </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>46</v>
-      </c>
-      <c r="N11">
-        <v>11</v>
-      </c>
-      <c r="O11">
-        <v>21</v>
-      </c>
-      <c r="P11">
-        <v>44</v>
-      </c>
-      <c r="Q11">
-        <v>53</v>
-      </c>
-      <c r="R11">
-        <v>59</v>
-      </c>
-      <c r="S11">
-        <v>50</v>
-      </c>
-      <c r="T11">
-        <v>52</v>
-      </c>
-      <c r="U11">
-        <v>55</v>
-      </c>
-      <c r="V11">
-        <v>58</v>
-      </c>
-      <c r="W11">
-        <v>64</v>
-      </c>
-      <c r="X11">
-        <v>50</v>
-      </c>
-      <c r="Y11">
-        <v>73</v>
-      </c>
-      <c r="Z11">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12">
-        <v>22</v>
-      </c>
-      <c r="C12">
-        <v>28</v>
-      </c>
-      <c r="D12">
-        <v>35</v>
-      </c>
-      <c r="E12">
-        <v>22</v>
-      </c>
-      <c r="F12">
-        <v>70</v>
-      </c>
-      <c r="G12">
-        <v>32</v>
-      </c>
-      <c r="H12">
-        <v>45</v>
-      </c>
-      <c r="I12">
-        <v>24</v>
-      </c>
-      <c r="J12">
-        <v>47</v>
-      </c>
-      <c r="K12">
-        <v>43</v>
-      </c>
-      <c r="L12">
-        <v>46</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>63</v>
-      </c>
-      <c r="O12">
-        <v>69</v>
-      </c>
-      <c r="P12">
-        <v>43</v>
-      </c>
-      <c r="Q12">
-        <v>64</v>
-      </c>
-      <c r="R12">
-        <v>66</v>
-      </c>
-      <c r="S12">
-        <v>43</v>
-      </c>
-      <c r="T12">
-        <v>58</v>
-      </c>
-      <c r="U12">
-        <v>62</v>
-      </c>
-      <c r="V12">
-        <v>70</v>
-      </c>
-      <c r="W12">
-        <v>66</v>
-      </c>
-      <c r="X12">
-        <v>66</v>
-      </c>
-      <c r="Y12">
-        <v>75</v>
-      </c>
-      <c r="Z12">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13">
-        <v>41</v>
-      </c>
-      <c r="C13">
-        <v>31</v>
-      </c>
-      <c r="D13">
-        <v>48</v>
-      </c>
-      <c r="E13">
-        <v>73</v>
-      </c>
-      <c r="F13">
-        <v>56</v>
-      </c>
-      <c r="G13">
-        <v>65</v>
-      </c>
-      <c r="H13">
-        <v>68</v>
-      </c>
-      <c r="I13">
-        <v>35</v>
-      </c>
-      <c r="J13">
-        <v>49</v>
-      </c>
-      <c r="K13">
-        <v>66</v>
-      </c>
-      <c r="L13">
-        <v>11</v>
-      </c>
-      <c r="M13">
-        <v>63</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
-        <v>27</v>
-      </c>
-      <c r="P13">
-        <v>71</v>
-      </c>
-      <c r="Q13">
-        <v>67</v>
-      </c>
-      <c r="R13">
-        <v>67</v>
-      </c>
-      <c r="S13">
-        <v>58</v>
-      </c>
-      <c r="T13">
-        <v>61</v>
-      </c>
-      <c r="U13">
-        <v>64</v>
-      </c>
-      <c r="V13">
-        <v>71</v>
-      </c>
-      <c r="W13">
-        <v>75</v>
-      </c>
-      <c r="X13">
-        <v>64</v>
-      </c>
-      <c r="Y13">
-        <v>74</v>
-      </c>
-      <c r="Z13">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14">
-        <v>48</v>
-      </c>
-      <c r="C14">
-        <v>35</v>
-      </c>
-      <c r="D14">
-        <v>54</v>
-      </c>
-      <c r="E14">
-        <v>72</v>
-      </c>
-      <c r="F14">
-        <v>56</v>
-      </c>
-      <c r="G14">
-        <v>74</v>
-      </c>
-      <c r="H14">
-        <v>76</v>
-      </c>
-      <c r="I14">
-        <v>35</v>
-      </c>
-      <c r="J14">
-        <v>53</v>
-      </c>
-      <c r="K14">
-        <v>61</v>
-      </c>
-      <c r="L14">
-        <v>21</v>
-      </c>
-      <c r="M14">
-        <v>69</v>
-      </c>
-      <c r="N14">
-        <v>27</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>73</v>
-      </c>
-      <c r="Q14">
-        <v>73</v>
-      </c>
-      <c r="R14">
-        <v>66</v>
-      </c>
-      <c r="S14">
-        <v>75</v>
-      </c>
-      <c r="T14">
-        <v>74</v>
-      </c>
-      <c r="U14">
-        <v>75</v>
-      </c>
-      <c r="V14">
-        <v>74</v>
-      </c>
-      <c r="W14">
-        <v>74</v>
-      </c>
-      <c r="X14">
-        <v>64</v>
-      </c>
-      <c r="Y14">
-        <v>78</v>
-      </c>
-      <c r="Z14">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>23</v>
-      </c>
-      <c r="C15">
-        <v>28</v>
-      </c>
-      <c r="D15">
-        <v>51</v>
-      </c>
-      <c r="E15">
-        <v>48</v>
-      </c>
-      <c r="F15">
-        <v>72</v>
-      </c>
-      <c r="G15">
-        <v>48</v>
-      </c>
-      <c r="H15">
-        <v>47</v>
-      </c>
-      <c r="I15">
-        <v>49</v>
-      </c>
-      <c r="J15">
-        <v>80</v>
-      </c>
-      <c r="K15">
-        <v>42</v>
-      </c>
-      <c r="L15">
-        <v>44</v>
-      </c>
-      <c r="M15">
-        <v>43</v>
-      </c>
-      <c r="N15">
-        <v>71</v>
-      </c>
-      <c r="O15">
-        <v>73</v>
-      </c>
-      <c r="P15">
-        <v>0</v>
-      </c>
-      <c r="Q15">
-        <v>52</v>
-      </c>
-      <c r="R15">
-        <v>64</v>
-      </c>
-      <c r="S15">
-        <v>51</v>
-      </c>
-      <c r="T15">
-        <v>58</v>
-      </c>
-      <c r="U15">
-        <v>62</v>
-      </c>
-      <c r="V15">
-        <v>63</v>
-      </c>
-      <c r="W15">
-        <v>63</v>
-      </c>
-      <c r="X15">
-        <v>50</v>
-      </c>
-      <c r="Y15">
-        <v>24</v>
-      </c>
-      <c r="Z15">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>20</v>
-      </c>
-      <c r="C16">
-        <v>47</v>
-      </c>
-      <c r="D16">
-        <v>73</v>
-      </c>
-      <c r="E16">
-        <v>48</v>
-      </c>
-      <c r="F16">
-        <v>73</v>
-      </c>
-      <c r="G16">
-        <v>55</v>
-      </c>
-      <c r="H16">
-        <v>63</v>
-      </c>
-      <c r="I16">
-        <v>54</v>
-      </c>
-      <c r="J16">
-        <v>64</v>
-      </c>
-      <c r="K16">
-        <v>57</v>
-      </c>
-      <c r="L16">
-        <v>53</v>
-      </c>
-      <c r="M16">
-        <v>64</v>
-      </c>
-      <c r="N16">
-        <v>67</v>
-      </c>
-      <c r="O16">
-        <v>73</v>
-      </c>
-      <c r="P16">
-        <v>52</v>
-      </c>
-      <c r="Q16">
-        <v>0</v>
-      </c>
-      <c r="R16">
-        <v>16</v>
-      </c>
-      <c r="S16">
-        <v>13</v>
-      </c>
-      <c r="T16">
-        <v>26</v>
-      </c>
-      <c r="U16">
-        <v>9</v>
-      </c>
-      <c r="V16">
-        <v>17</v>
-      </c>
-      <c r="W16">
-        <v>18</v>
-      </c>
-      <c r="X16">
-        <v>40</v>
-      </c>
-      <c r="Y16">
-        <v>11</v>
-      </c>
-      <c r="Z16">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>33</v>
-      </c>
-      <c r="C17">
-        <v>65</v>
-      </c>
-      <c r="D17">
-        <v>64</v>
-      </c>
-      <c r="E17">
-        <v>53</v>
-      </c>
-      <c r="F17">
-        <v>53</v>
-      </c>
-      <c r="G17">
-        <v>55</v>
-      </c>
-      <c r="H17">
-        <v>72</v>
-      </c>
-      <c r="I17">
-        <v>59</v>
-      </c>
-      <c r="J17">
-        <v>55</v>
-      </c>
-      <c r="K17">
-        <v>68</v>
-      </c>
-      <c r="L17">
-        <v>59</v>
-      </c>
-      <c r="M17">
-        <v>66</v>
-      </c>
-      <c r="N17">
-        <v>67</v>
-      </c>
-      <c r="O17">
-        <v>66</v>
-      </c>
-      <c r="P17">
-        <v>64</v>
-      </c>
-      <c r="Q17">
-        <v>16</v>
-      </c>
-      <c r="R17">
-        <v>0</v>
-      </c>
-      <c r="S17">
-        <v>12</v>
-      </c>
-      <c r="T17">
-        <v>27</v>
-      </c>
-      <c r="U17">
-        <v>23</v>
-      </c>
-      <c r="V17">
-        <v>32</v>
-      </c>
-      <c r="W17">
-        <v>34</v>
-      </c>
-      <c r="X17">
-        <v>38</v>
-      </c>
-      <c r="Y17">
-        <v>16</v>
-      </c>
-      <c r="Z17">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>18</v>
-      </c>
-      <c r="C18">
-        <v>49</v>
-      </c>
-      <c r="D18">
-        <v>74</v>
-      </c>
-      <c r="E18">
-        <v>26</v>
-      </c>
-      <c r="F18">
-        <v>67</v>
-      </c>
-      <c r="G18">
-        <v>26</v>
-      </c>
-      <c r="H18">
-        <v>58</v>
-      </c>
-      <c r="I18">
-        <v>54</v>
-      </c>
-      <c r="J18">
-        <v>71</v>
-      </c>
-      <c r="K18">
-        <v>46</v>
-      </c>
-      <c r="L18">
-        <v>50</v>
-      </c>
-      <c r="M18">
-        <v>43</v>
-      </c>
-      <c r="N18">
-        <v>58</v>
-      </c>
-      <c r="O18">
-        <v>75</v>
-      </c>
-      <c r="P18">
-        <v>51</v>
-      </c>
-      <c r="Q18">
-        <v>13</v>
-      </c>
-      <c r="R18">
-        <v>12</v>
-      </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18">
-        <v>11</v>
-      </c>
-      <c r="U18">
-        <v>29</v>
-      </c>
-      <c r="V18">
-        <v>35</v>
-      </c>
-      <c r="W18">
-        <v>34</v>
-      </c>
-      <c r="X18">
-        <v>52</v>
-      </c>
-      <c r="Y18">
-        <v>17</v>
-      </c>
-      <c r="Z18">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>28</v>
-      </c>
-      <c r="C19">
-        <v>58</v>
-      </c>
-      <c r="D19">
-        <v>76</v>
-      </c>
-      <c r="E19">
-        <v>46</v>
-      </c>
-      <c r="F19">
-        <v>62</v>
-      </c>
-      <c r="G19">
-        <v>37</v>
-      </c>
-      <c r="H19">
-        <v>57</v>
-      </c>
-      <c r="I19">
-        <v>60</v>
-      </c>
-      <c r="J19">
-        <v>69</v>
-      </c>
-      <c r="K19">
-        <v>57</v>
-      </c>
-      <c r="L19">
-        <v>52</v>
-      </c>
-      <c r="M19">
-        <v>58</v>
-      </c>
-      <c r="N19">
-        <v>61</v>
-      </c>
-      <c r="O19">
-        <v>74</v>
-      </c>
-      <c r="P19">
-        <v>58</v>
-      </c>
-      <c r="Q19">
-        <v>26</v>
-      </c>
-      <c r="R19">
-        <v>27</v>
-      </c>
-      <c r="S19">
-        <v>11</v>
-      </c>
-      <c r="T19">
-        <v>0</v>
-      </c>
-      <c r="U19">
-        <v>32</v>
-      </c>
-      <c r="V19">
-        <v>40</v>
-      </c>
-      <c r="W19">
-        <v>39</v>
-      </c>
-      <c r="X19">
-        <v>56</v>
-      </c>
-      <c r="Y19">
-        <v>45</v>
-      </c>
-      <c r="Z19">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>22</v>
-      </c>
-      <c r="C20">
-        <v>49</v>
-      </c>
-      <c r="D20">
-        <v>70</v>
-      </c>
-      <c r="E20">
-        <v>50</v>
-      </c>
-      <c r="F20">
-        <v>62</v>
-      </c>
-      <c r="G20">
-        <v>47</v>
-      </c>
-      <c r="H20">
-        <v>60</v>
-      </c>
-      <c r="I20">
-        <v>60</v>
-      </c>
-      <c r="J20">
-        <v>73</v>
-      </c>
-      <c r="K20">
-        <v>63</v>
-      </c>
-      <c r="L20">
-        <v>55</v>
-      </c>
-      <c r="M20">
-        <v>62</v>
-      </c>
-      <c r="N20">
-        <v>64</v>
-      </c>
-      <c r="O20">
-        <v>75</v>
-      </c>
-      <c r="P20">
-        <v>62</v>
-      </c>
-      <c r="Q20">
-        <v>9</v>
-      </c>
-      <c r="R20">
-        <v>23</v>
-      </c>
-      <c r="S20">
-        <v>29</v>
-      </c>
-      <c r="T20">
-        <v>32</v>
-      </c>
-      <c r="U20">
-        <v>0</v>
-      </c>
-      <c r="V20">
-        <v>8</v>
-      </c>
-      <c r="W20">
-        <v>9</v>
-      </c>
-      <c r="X20">
-        <v>27</v>
-      </c>
-      <c r="Y20">
-        <v>33</v>
-      </c>
-      <c r="Z20">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>30</v>
-      </c>
-      <c r="C21">
-        <v>64</v>
-      </c>
-      <c r="D21">
-        <v>47</v>
-      </c>
-      <c r="E21">
-        <v>48</v>
-      </c>
-      <c r="F21">
-        <v>73</v>
-      </c>
-      <c r="G21">
-        <v>49</v>
-      </c>
-      <c r="H21">
-        <v>63</v>
-      </c>
-      <c r="I21">
-        <v>63</v>
-      </c>
-      <c r="J21">
-        <v>75</v>
-      </c>
-      <c r="K21">
-        <v>64</v>
-      </c>
-      <c r="L21">
-        <v>58</v>
-      </c>
-      <c r="M21">
-        <v>70</v>
-      </c>
-      <c r="N21">
-        <v>71</v>
-      </c>
-      <c r="O21">
-        <v>74</v>
-      </c>
-      <c r="P21">
-        <v>63</v>
-      </c>
-      <c r="Q21">
-        <v>17</v>
-      </c>
-      <c r="R21">
-        <v>32</v>
-      </c>
-      <c r="S21">
-        <v>35</v>
-      </c>
-      <c r="T21">
-        <v>40</v>
-      </c>
-      <c r="U21">
-        <v>8</v>
-      </c>
-      <c r="V21">
-        <v>0</v>
-      </c>
-      <c r="W21">
-        <v>19</v>
-      </c>
-      <c r="X21">
-        <v>23</v>
-      </c>
-      <c r="Y21">
-        <v>60</v>
-      </c>
-      <c r="Z21">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>31</v>
-      </c>
-      <c r="C22">
-        <v>55</v>
-      </c>
-      <c r="D22">
-        <v>78</v>
-      </c>
-      <c r="E22">
-        <v>54</v>
-      </c>
-      <c r="F22">
-        <v>68</v>
-      </c>
-      <c r="G22">
-        <v>53</v>
-      </c>
-      <c r="H22">
-        <v>67</v>
-      </c>
-      <c r="I22">
-        <v>63</v>
-      </c>
-      <c r="J22">
-        <v>72</v>
-      </c>
-      <c r="K22">
-        <v>57</v>
-      </c>
-      <c r="L22">
-        <v>64</v>
-      </c>
-      <c r="M22">
-        <v>66</v>
-      </c>
-      <c r="N22">
-        <v>75</v>
-      </c>
-      <c r="O22">
-        <v>74</v>
-      </c>
-      <c r="P22">
-        <v>63</v>
-      </c>
-      <c r="Q22">
-        <v>18</v>
-      </c>
-      <c r="R22">
-        <v>34</v>
-      </c>
-      <c r="S22">
-        <v>34</v>
-      </c>
-      <c r="T22">
-        <v>39</v>
-      </c>
-      <c r="U22">
-        <v>9</v>
-      </c>
-      <c r="V22">
-        <v>19</v>
-      </c>
-      <c r="W22">
-        <v>0</v>
-      </c>
-      <c r="X22">
-        <v>43</v>
-      </c>
-      <c r="Y22">
-        <v>49</v>
-      </c>
-      <c r="Z22">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>45</v>
-      </c>
-      <c r="C23">
-        <v>53</v>
-      </c>
-      <c r="D23">
-        <v>35</v>
-      </c>
-      <c r="E23">
-        <v>45</v>
-      </c>
-      <c r="F23">
-        <v>45</v>
-      </c>
-      <c r="G23">
-        <v>39</v>
-      </c>
-      <c r="H23">
-        <v>55</v>
-      </c>
-      <c r="I23">
-        <v>56</v>
-      </c>
-      <c r="J23">
-        <v>49</v>
-      </c>
-      <c r="K23">
-        <v>51</v>
-      </c>
-      <c r="L23">
-        <v>50</v>
-      </c>
-      <c r="M23">
-        <v>66</v>
-      </c>
-      <c r="N23">
-        <v>64</v>
-      </c>
-      <c r="O23">
-        <v>64</v>
-      </c>
-      <c r="P23">
-        <v>50</v>
-      </c>
-      <c r="Q23">
-        <v>40</v>
-      </c>
-      <c r="R23">
-        <v>38</v>
-      </c>
-      <c r="S23">
-        <v>52</v>
-      </c>
-      <c r="T23">
-        <v>56</v>
-      </c>
-      <c r="U23">
-        <v>27</v>
-      </c>
-      <c r="V23">
-        <v>23</v>
-      </c>
-      <c r="W23">
-        <v>43</v>
-      </c>
-      <c r="X23">
-        <v>0</v>
-      </c>
-      <c r="Y23">
-        <v>10</v>
-      </c>
-      <c r="Z23">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>35</v>
-      </c>
-      <c r="C24">
-        <v>69</v>
-      </c>
-      <c r="D24">
-        <v>76</v>
-      </c>
-      <c r="E24">
-        <v>65</v>
-      </c>
-      <c r="F24">
-        <v>59</v>
-      </c>
-      <c r="G24">
-        <v>74</v>
-      </c>
-      <c r="H24">
-        <v>78</v>
-      </c>
-      <c r="I24">
-        <v>72</v>
-      </c>
-      <c r="J24">
-        <v>75</v>
-      </c>
-      <c r="K24">
-        <v>77</v>
-      </c>
-      <c r="L24">
-        <v>73</v>
-      </c>
-      <c r="M24">
-        <v>75</v>
-      </c>
-      <c r="N24">
-        <v>74</v>
-      </c>
-      <c r="O24">
-        <v>78</v>
-      </c>
-      <c r="P24">
-        <v>24</v>
-      </c>
-      <c r="Q24">
-        <v>11</v>
-      </c>
-      <c r="R24">
-        <v>16</v>
-      </c>
-      <c r="S24">
-        <v>17</v>
-      </c>
-      <c r="T24">
-        <v>45</v>
-      </c>
-      <c r="U24">
-        <v>33</v>
-      </c>
-      <c r="V24">
-        <v>60</v>
-      </c>
-      <c r="W24">
-        <v>49</v>
-      </c>
-      <c r="X24">
-        <v>10</v>
-      </c>
-      <c r="Y24">
-        <v>0</v>
-      </c>
-      <c r="Z24">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>62</v>
-      </c>
-      <c r="C25">
-        <v>63</v>
-      </c>
-      <c r="D25">
-        <v>15</v>
-      </c>
-      <c r="E25">
-        <v>49</v>
-      </c>
-      <c r="F25">
-        <v>43</v>
-      </c>
-      <c r="G25">
-        <v>27</v>
-      </c>
-      <c r="H25">
-        <v>56</v>
-      </c>
-      <c r="I25">
-        <v>62</v>
-      </c>
-      <c r="J25">
-        <v>58</v>
-      </c>
-      <c r="K25">
-        <v>62</v>
-      </c>
-      <c r="L25">
-        <v>69</v>
-      </c>
-      <c r="M25">
-        <v>70</v>
-      </c>
-      <c r="N25">
-        <v>69</v>
-      </c>
-      <c r="O25">
-        <v>73</v>
-      </c>
-      <c r="P25">
-        <v>78</v>
-      </c>
-      <c r="Q25">
-        <v>47</v>
-      </c>
-      <c r="R25">
-        <v>44</v>
-      </c>
-      <c r="S25">
-        <v>61</v>
-      </c>
-      <c r="T25">
-        <v>65</v>
-      </c>
-      <c r="U25">
-        <v>30</v>
-      </c>
-      <c r="V25">
-        <v>14</v>
-      </c>
-      <c r="W25">
-        <v>58</v>
-      </c>
-      <c r="X25">
-        <v>11</v>
-      </c>
-      <c r="Y25">
-        <v>32</v>
-      </c>
-      <c r="Z25">
         <v>0</v>
       </c>
     </row>

</xml_diff>